<commit_message>
face_snapshot: apply AC overview review decisions
</commit_message>
<xml_diff>
--- a/branch_diff/face_snapshot-new/ac侧提交概览.xlsx
+++ b/branch_diff/face_snapshot-new/ac侧提交概览.xlsx
@@ -66,7 +66,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:dimension ref="A1:O31"/>
+  <ns0:dimension ref="A1:O30"/>
   <ns0:cols>
     <ns0:col min="1" max="1" width="9" customWidth="1"/>
     <ns0:col min="2" max="2" width="15" customWidth="1"/>
@@ -163,134 +163,142 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="2">
-      <ns0:c r="A2" s="2">
+      <ns0:c r="A2" s="0">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="B2" s="2" t="inlineStr">
+      <ns0:c r="B2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2024-11-04</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C2" s="2" t="inlineStr">
+      <ns0:c r="C2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">531e6162</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D2" s="2" t="inlineStr">
+      <ns0:c r="D2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[all] cap|face_snapshot: support face_snapshot data model</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E2" s="2" t="inlineStr">
+      <ns0:c r="E2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">集中合入</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F2" s="2" t="inlineStr">
+      <ns0:c r="F2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">I6a975f02a9b2b97d9c18dc01441b846baa9fe720</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G2" s="2" t="inlineStr">
+      <ns0:c r="G2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">建立人脸快照的数据模型与默认配置，加入规则、图片、容量和存储头文件，供后续识别及管理接口使用。</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="H2" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I2" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J2" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K2" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L2" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M2" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N2" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O2" s="2" t="inlineStr">
+      <ns0:c r="H2" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I2" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N2" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O2" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
       </ns0:c>
     </ns0:row>
     <ns0:row r="3">
-      <ns0:c r="A3" s="2">
+      <ns0:c r="A3" s="0">
         <ns0:v>2</ns0:v>
       </ns0:c>
-      <ns0:c r="B3" s="2" t="inlineStr">
+      <ns0:c r="B3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2024-11-13</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C3" s="2" t="inlineStr">
+      <ns0:c r="C3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">98a66a72</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D3" s="2" t="inlineStr">
+      <ns0:c r="D3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[all] cap|support face_recognition</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E3" s="2" t="inlineStr">
+      <ns0:c r="E3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">集中合入</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F3" s="2" t="inlineStr">
+      <ns0:c r="F3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Ib2cba2be7471709a3188a2c0c9ded507f13961cb</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G3" s="2" t="inlineStr">
+      <ns0:c r="G3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">加入人脸识别主体实现，涵盖特征管理、相似度搜索、人脸信息存储与控制接口，是 AC 侧后续修复的基础。</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="H3" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I3" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J3" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K3" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O3" s="2" t="inlineStr">
+      <ns0:c r="H3" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I3" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N3" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O3" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -317,7 +325,7 @@
       </ns0:c>
       <ns0:c r="E4" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F4" s="0" t="inlineStr">
@@ -435,134 +443,142 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="6">
-      <ns0:c r="A6" s="2">
+      <ns0:c r="A6" s="0">
         <ns0:v>5</ns0:v>
       </ns0:c>
-      <ns0:c r="B6" s="2" t="inlineStr">
+      <ns0:c r="B6" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2024-12-17</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C6" s="2" t="inlineStr">
+      <ns0:c r="C6" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">906e6b5e</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D6" s="2" t="inlineStr">
+      <ns0:c r="D6" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[all] cap:调整日志接口宏定义适配日志分类(3/4)-patch</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E6" s="2" t="inlineStr">
+      <ns0:c r="E6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">098日志宏相关</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ia124c27c4c2fa84d670196a76da1c34124f03320</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">适配日志分类接口，将人脸存储头文件中的日志宏调整为新形式；原系列横跨其他模块。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H6" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I6" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O6" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" s="0">
+        <ns0:v>6</ns0:v>
+      </ns0:c>
+      <ns0:c r="B7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2025-06-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">3f74974b</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[all]change manufacturer name in NVMP platform code</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">代码优化</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ia124c27c4c2fa84d670196a76da1c34124f03320</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">适配日志分类接口，将人脸存储头文件中的日志宏调整为新形式；原系列横跨其他模块。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H6" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I6" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J6" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K6" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" s="2">
-        <ns0:v>6</ns0:v>
-      </ns0:c>
-      <ns0:c r="B7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2025-06-05</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">3f74974b</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[all]change manufacturer name in NVMP platform code</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">代码优化</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F7" s="2" t="inlineStr">
+      <ns0:c r="F7" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Idee1613673382383f22025fcefa25ac5fc31362d</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G7" s="2" t="inlineStr">
+      <ns0:c r="G7" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">将人脸快照相关文件头中的厂商名称与版权标识更新为新的公司名称；属于平台批量名称修改。</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="H7" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I7" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J7" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K7" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O7" s="2" t="inlineStr">
+      <ns0:c r="H7" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I7" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N7" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O7" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -798,7 +814,7 @@
       </ns0:c>
       <ns0:c r="E11" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F11" s="0" t="inlineStr">
@@ -869,7 +885,7 @@
       </ns0:c>
       <ns0:c r="E12" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">配置调整</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F12" s="0" t="inlineStr">
@@ -940,7 +956,7 @@
       </ns0:c>
       <ns0:c r="E13" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F13" s="0" t="inlineStr">
@@ -1011,7 +1027,7 @@
       </ns0:c>
       <ns0:c r="E14" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
+          <ns0:t xml:space="preserve">Bug修复,有对标提交</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F14" s="2" t="inlineStr">
@@ -1021,7 +1037,7 @@
       </ns0:c>
       <ns0:c r="G14" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">修正人脸控制与统计中的多处问题，涉及旧人脸删除、状态传递、HUB 相关处理及统计队列边界。</ns0:t>
+          <ns0:t xml:space="preserve">与 BC 99edff3d 同 Change-Id，六项修复目标一致，均处理 HUB 配置缓存、合并旧人脸删除、队列校验及库满覆盖通知；补丁不逐行相同。AC 的 HUB 告警保留 pushable:0，内部删除额外清理陌生人历史，检测入口兼容 PSS；BC 原补丁沿用无 pushable 的 HUB 格式与自身检测入口。需按最终代码核对这些差异。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H14" s="2">
@@ -1078,7 +1094,7 @@
       </ns0:c>
       <ns0:c r="E15" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F15" s="0" t="inlineStr">
@@ -1129,67 +1145,67 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="16">
-      <ns0:c r="A16" s="2">
+      <ns0:c r="A16" s="0">
         <ns0:v>15</ns0:v>
       </ns0:c>
-      <ns0:c r="B16" s="2" t="inlineStr">
+      <ns0:c r="B16" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2026-01-16</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C16" s="2" t="inlineStr">
+      <ns0:c r="C16" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">91713aef</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D16" s="2" t="inlineStr">
+      <ns0:c r="D16" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[CAP]face_control:fix face_snapshot config[1/2]</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E16" s="2" t="inlineStr">
+      <ns0:c r="E16" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">配置修复</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F16" s="2" t="inlineStr">
+      <ns0:c r="F16" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Iedc5cdd41603571b67902f89c0f315515ee2b2fa</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">为历史图片保存配置加入迁移修复入口，在需要时将旧的 save_pic 配置关闭；是否启用依赖编译宏及系列配套。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H16" s="2">
+      <ns0:c r="G16" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">修复旧 save_pic 配置的入口受单侧 FIX_FSS_PIC_CFG 编译宏限制；目标分支虽有对应函数，宏的实际启用和系列配套仍需复核。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H16" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I16" s="0">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="I16" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J16" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K16" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O16" s="2" t="inlineStr">
+      <ns0:c r="J16" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K16" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L16" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M16" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N16" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O16" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -1216,7 +1232,7 @@
       </ns0:c>
       <ns0:c r="E17" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F17" s="0" t="inlineStr">
@@ -1287,7 +1303,7 @@
       </ns0:c>
       <ns0:c r="E18" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">跨模块修复</ns0:t>
+          <ns0:t xml:space="preserve">bug修复，hub相关，需谨慎</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F18" s="2" t="inlineStr">
@@ -1354,7 +1370,7 @@
       </ns0:c>
       <ns0:c r="E19" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">编译修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F19" s="0" t="inlineStr">
@@ -1406,7 +1422,7 @@
     </ns0:row>
     <ns0:row r="20">
       <ns0:c r="A20" s="0">
-        <ns0:v>19</ns0:v>
+        <ns0:v>20</ns0:v>
       </ns0:c>
       <ns0:c r="B20" s="0" t="inlineStr">
         <ns0:is>
@@ -1415,7 +1431,7 @@
       </ns0:c>
       <ns0:c r="C20" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">6f4f42d7</ns0:t>
+          <ns0:t xml:space="preserve">2fc6094a</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D20" s="0" t="inlineStr">
@@ -1435,7 +1451,7 @@
       </ns0:c>
       <ns0:c r="G20" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">优化 face_info 文件头和记录的校验流程，避免异常数据进入加载路径，并修复相关存储判断。</ns0:t>
+          <ns0:t xml:space="preserve">继续修正 face_info 文件校验流程与异常处理；与前一笔及 BC 对应补丁属于同一问题链。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H20" s="0">
@@ -1476,138 +1492,138 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="21">
-      <ns0:c r="A21" s="0">
-        <ns0:v>20</ns0:v>
-      </ns0:c>
-      <ns0:c r="B21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2026-05-06</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2fc6094a</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[all] fss: Optimize the validation process for the face_info file and fix a bug</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">I86979829357c6d3f5b19b81593207a4980e05bd6</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">继续修正 face_info 文件校验流程与异常处理；与前一笔及 BC 对应补丁属于同一问题链。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H21" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I21" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N21" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O21" s="0" t="inlineStr">
+      <ns0:c r="A21" s="2">
+        <ns0:v>21</ns0:v>
+      </ns0:c>
+      <ns0:c r="B21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-05-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">7bbf5e9a</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[cap]fss:fix compile error and standardize code</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">跨模块修复</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I377a261c1bf79959b51effbdfcf8cb9b55ed48c7</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">注册人脸快照供 libfss 使用的回调接口并规范代码；关联 NVMP、AVTS、NSD 等仓库的接口和消费者。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H21" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="I21" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="J21" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K21" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N21" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O21" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
       </ns0:c>
     </ns0:row>
     <ns0:row r="22">
-      <ns0:c r="A22" s="2">
-        <ns0:v>21</ns0:v>
-      </ns0:c>
-      <ns0:c r="B22" s="2" t="inlineStr">
+      <ns0:c r="A22" s="0">
+        <ns0:v>22</ns0:v>
+      </ns0:c>
+      <ns0:c r="B22" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2026-05-07</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">7bbf5e9a</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[cap]fss:fix compile error and standardize code</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">跨模块修复</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">I377a261c1bf79959b51effbdfcf8cb9b55ed48c7</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">注册人脸快照供 libfss 使用的回调接口并规范代码；关联 NVMP、AVTS、NSD 等仓库的接口和消费者。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H22" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I22" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J22" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K22" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N22" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O22" s="2" t="inlineStr">
+      <ns0:c r="C22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">c9e47da4</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[cap]face_snapshot:correct the storage path of fss</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I857ac9930f05ab869cc112f8df0a6b6136b91723</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">修正人脸快照存储路径常量，避免数据写入错误目录。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H22" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I22" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N22" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O22" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -1615,36 +1631,36 @@
     </ns0:row>
     <ns0:row r="23">
       <ns0:c r="A23" s="0">
-        <ns0:v>22</ns0:v>
+        <ns0:v>23</ns0:v>
       </ns0:c>
       <ns0:c r="B23" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-05-07</ns0:t>
+          <ns0:t xml:space="preserve">2026-05-11</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C23" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">c9e47da4</ns0:t>
+          <ns0:t xml:space="preserve">593c131a</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">[cap]face_snapshot:correct the storage path of fss</ns0:t>
+          <ns0:t xml:space="preserve">[CAP] merge (non-core)commit (interface capability variable) from nvmp_release_1.8.1_secure_enhance_250707 to other branch (3/5)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E23" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">配置修复</ns0:t>
+          <ns0:t xml:space="preserve">特殊提交</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F23" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">I857ac9930f05ab869cc112f8df0a6b6136b91723</ns0:t>
+          <ns0:t xml:space="preserve">I532bda5ddb70bb9c1d7f6c0f6be0877606743bb9</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">修正人脸快照存储路径常量，避免数据写入错误目录。</ns0:t>
+          <ns0:t xml:space="preserve">把旧版本的接口能力变量与 DS 模板适配代码整合到当前分支；face_snapshot 只占原跨模块提交的一部分。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H23" s="0">
@@ -1686,36 +1702,36 @@
     </ns0:row>
     <ns0:row r="24">
       <ns0:c r="A24" s="0">
-        <ns0:v>23</ns0:v>
+        <ns0:v>24</ns0:v>
       </ns0:c>
       <ns0:c r="B24" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-05-11</ns0:t>
+          <ns0:t xml:space="preserve">2026-05-15</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C24" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">593c131a</ns0:t>
+          <ns0:t xml:space="preserve">d86eea00</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D24" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">[CAP] merge (non-core)commit (interface capability variable) from nvmp_release_1.8.1_secure_enhance_250707 to other branch (3/5)</ns0:t>
+          <ns0:t xml:space="preserve">[all]face_snapshot|usr_cfg_conv:resolve the DOS attack caused by the connect interface(3/4)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E24" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">分支合并提交</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F24" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">I532bda5ddb70bb9c1d7f6c0f6be0877606743bb9</ns0:t>
+          <ns0:t xml:space="preserve">I37a170e9d0d770563ab55e459c6fea66683a01c6</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">把旧版本的接口能力变量与 DS 模板适配代码整合到当前分支；face_snapshot 只占原跨模块提交的一部分。</ns0:t>
+          <ns0:t xml:space="preserve">修正连接接口中 Base64 解码的输出容量初始化，限制解码写入范围以避免拒绝服务问题。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H24" s="0">
@@ -1757,36 +1773,36 @@
     </ns0:row>
     <ns0:row r="25">
       <ns0:c r="A25" s="0">
-        <ns0:v>24</ns0:v>
+        <ns0:v>25</ns0:v>
       </ns0:c>
       <ns0:c r="B25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-05-15</ns0:t>
+          <ns0:t xml:space="preserve">2026-06-29</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">d86eea00</ns0:t>
+          <ns0:t xml:space="preserve">f76e5b84</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">[all]face_snapshot|usr_cfg_conv:resolve the DOS attack caused by the connect interface(3/4)</ns0:t>
+          <ns0:t xml:space="preserve">[all] fss: fixed - face latest time update anomaly.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">安全修复</ns0:t>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">I37a170e9d0d770563ab55e459c6fea66683a01c6</ns0:t>
+          <ns0:t xml:space="preserve">I752abbfd4cb70c12b4afbe03096451336886e985</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">修正连接接口中 Base64 解码的输出容量初始化，限制解码写入范围以避免拒绝服务问题。</ns0:t>
+          <ns0:t xml:space="preserve">修正人脸最新出现时间的更新条件，避免事件记录停留在旧时间。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H25" s="0">
@@ -1827,209 +1843,205 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="26">
-      <ns0:c r="A26" s="0">
-        <ns0:v>25</ns0:v>
-      </ns0:c>
-      <ns0:c r="B26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2026-06-29</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">f76e5b84</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[all] fss: fixed - face latest time update anomaly.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Bug修复</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">I752abbfd4cb70c12b4afbe03096451336886e985</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">修正人脸最新出现时间的更新条件，避免事件记录停留在旧时间。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H26" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I26" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N26" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O26" s="0" t="inlineStr">
+      <ns0:c r="A26" s="2">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="B26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-06-26</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">1ab52989</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[ALL] telemetry:telemetry support face recognition(2/3)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">功能扩充</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Ie856cee55e225d820d93afd90b143a7f575e585c</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">增加人脸识别遥测数据、采集回调和 getFaceTelemetryInfo 接口，供外部模块读取识别统计；属于跨仓系列。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H26" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="I26" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="J26" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K26" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N26" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O26" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
       </ns0:c>
     </ns0:row>
     <ns0:row r="27">
-      <ns0:c r="A27" s="2">
-        <ns0:v>26</ns0:v>
-      </ns0:c>
-      <ns0:c r="B27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2026-06-26</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">1ab52989</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[ALL] telemetry:telemetry support face recognition(2/3)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">功能扩充</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Ie856cee55e225d820d93afd90b143a7f575e585c</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">增加人脸识别遥测数据、采集回调和 getFaceTelemetryInfo 接口，供外部模块读取识别统计；属于跨仓系列。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H27" s="2">
+      <ns0:c r="A27" s="0">
+        <ns0:v>27</ns0:v>
+      </ns0:c>
+      <ns0:c r="B27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-07-13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">ebb0da21</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[ALL] face_snapshot: Fix non-standard code for telemetry support of face recognition</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">编译修复</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I7dd93f69b756a90ae4b67e4f2573f4c1d20d2ba5</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">修正人脸识别遥测代码的宏边界、空参数返回及接口注册保护，使可选遥测配置下的代码规范且可编译。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H27" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I27" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" s="2">
+        <ns0:v>28</ns0:v>
+      </ns0:c>
+      <ns0:c r="B28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-07-27</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">dd2600fb</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap:Add camera log (3/4)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">跨模块功能</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I546ddacdc3c963356cab324458b2e295a1b62e66</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">在人脸快照配置链中接入摄像机操作日志，记录相关配置动作；属于跨模块系列的 CAP 部分。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H28" s="2">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="I27" s="2">
+      <ns0:c r="I28" s="2">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="J27" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K27" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O27" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" s="0">
-        <ns0:v>27</ns0:v>
-      </ns0:c>
-      <ns0:c r="B28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2026-07-13</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">ebb0da21</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[ALL] face_snapshot: Fix non-standard code for telemetry support of face recognition</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">编译修复</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">I7dd93f69b756a90ae4b67e4f2573f4c1d20d2ba5</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">修正人脸识别遥测代码的宏边界、空参数返回及接口注册保护，使可选遥测配置下的代码规范且可编译。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H28" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I28" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N28" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O28" s="0" t="inlineStr">
+      <ns0:c r="J28" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K28" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N28" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O28" s="2" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -2037,21 +2049,21 @@
     </ns0:row>
     <ns0:row r="29">
       <ns0:c r="A29" s="2">
-        <ns0:v>28</ns0:v>
+        <ns0:v>29</ns0:v>
       </ns0:c>
       <ns0:c r="B29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-07-27</ns0:t>
+          <ns0:t xml:space="preserve">2026-08-14</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">dd2600fb</ns0:t>
+          <ns0:t xml:space="preserve">14378dec</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap:Add camera log (3/4)</ns0:t>
+          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap: modify pre_set method(2/2)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E29" s="2" t="inlineStr">
@@ -2061,12 +2073,12 @@
       </ns0:c>
       <ns0:c r="F29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">I546ddacdc3c963356cab324458b2e295a1b62e66</ns0:t>
+          <ns0:t xml:space="preserve">Iaf8476f2cb5fc327339218e1cf59a10f865c9bd7</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">在人脸快照配置链中接入摄像机操作日志，记录相关配置动作；属于跨模块系列的 CAP 部分。</ns0:t>
+          <ns0:t xml:space="preserve">调整摄像机操作日志相关配置的预设置方法，使配置变更和日志链一致；需结合系列其他模块评审。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H29" s="2">
@@ -2103,144 +2115,77 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="30">
-      <ns0:c r="A30" s="2">
-        <ns0:v>29</ns0:v>
-      </ns0:c>
-      <ns0:c r="B30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2026-08-14</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">14378dec</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap: modify pre_set method(2/2)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">跨模块功能</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">Iaf8476f2cb5fc327339218e1cf59a10f865c9bd7</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">调整摄像机操作日志相关配置的预设置方法，使配置变更和日志链一致；需结合系列其他模块评审。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H30" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I30" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J30" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K30" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O30" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="31">
-      <ns0:c r="A31" s="0">
+      <ns0:c r="A30" s="0">
         <ns0:v>30</ns0:v>
       </ns0:c>
-      <ns0:c r="B31" s="0" t="inlineStr">
+      <ns0:c r="B30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2026-09-21</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C31" s="0" t="inlineStr">
+      <ns0:c r="C30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">178f33f6</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D31" s="0" t="inlineStr">
+      <ns0:c r="D30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[all]cap:Fixed the error in determining the fd in err_exit</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E31" s="0" t="inlineStr">
+      <ns0:c r="E30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Bug修复</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F31" s="0" t="inlineStr">
+      <ns0:c r="F30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Ia28fea5b1b63f8146d857ecbcff25f66326e1041</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G31" s="0" t="inlineStr">
+      <ns0:c r="G30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">修正 PSS 图片复制函数错误退出时的文件描述符判断，按原提交条件关闭已打开的源文件与目标文件。</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="H31" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I31" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N31" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O31" s="0" t="inlineStr">
+      <ns0:c r="H30" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I30" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J30" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K30" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L30" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M30" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N30" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O30" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>
-  <ns0:autoFilter ref="A1:O31"/>
+  <ns0:autoFilter ref="A1:O30"/>
 </ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
face_snapshot: canonicalize AC overview on develop branch
</commit_message>
<xml_diff>
--- a/branch_diff/face_snapshot-new/ac侧提交概览.xlsx
+++ b/branch_diff/face_snapshot-new/ac侧提交概览.xlsx
@@ -66,7 +66,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:dimension ref="A1:O30"/>
+  <ns0:dimension ref="A1:O31"/>
   <ns0:cols>
     <ns0:col min="1" max="1" width="9" customWidth="1"/>
     <ns0:col min="2" max="2" width="15" customWidth="1"/>
@@ -1422,7 +1422,7 @@
     </ns0:row>
     <ns0:row r="20">
       <ns0:c r="A20" s="0">
-        <ns0:v>20</ns0:v>
+        <ns0:v>19</ns0:v>
       </ns0:c>
       <ns0:c r="B20" s="0" t="inlineStr">
         <ns0:is>
@@ -1493,7 +1493,7 @@
     </ns0:row>
     <ns0:row r="21">
       <ns0:c r="A21" s="2">
-        <ns0:v>21</ns0:v>
+        <ns0:v>20</ns0:v>
       </ns0:c>
       <ns0:c r="B21" s="2" t="inlineStr">
         <ns0:is>
@@ -1560,7 +1560,7 @@
     </ns0:row>
     <ns0:row r="22">
       <ns0:c r="A22" s="0">
-        <ns0:v>22</ns0:v>
+        <ns0:v>21</ns0:v>
       </ns0:c>
       <ns0:c r="B22" s="0" t="inlineStr">
         <ns0:is>
@@ -1631,7 +1631,7 @@
     </ns0:row>
     <ns0:row r="23">
       <ns0:c r="A23" s="0">
-        <ns0:v>23</ns0:v>
+        <ns0:v>22</ns0:v>
       </ns0:c>
       <ns0:c r="B23" s="0" t="inlineStr">
         <ns0:is>
@@ -1702,7 +1702,7 @@
     </ns0:row>
     <ns0:row r="24">
       <ns0:c r="A24" s="0">
-        <ns0:v>24</ns0:v>
+        <ns0:v>23</ns0:v>
       </ns0:c>
       <ns0:c r="B24" s="0" t="inlineStr">
         <ns0:is>
@@ -1773,7 +1773,7 @@
     </ns0:row>
     <ns0:row r="25">
       <ns0:c r="A25" s="0">
-        <ns0:v>25</ns0:v>
+        <ns0:v>24</ns0:v>
       </ns0:c>
       <ns0:c r="B25" s="0" t="inlineStr">
         <ns0:is>
@@ -1782,7 +1782,7 @@
       </ns0:c>
       <ns0:c r="C25" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">f76e5b84</ns0:t>
+          <ns0:t xml:space="preserve">5400834e</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D25" s="0" t="inlineStr">
@@ -1844,16 +1844,16 @@
     </ns0:row>
     <ns0:row r="26">
       <ns0:c r="A26" s="2">
-        <ns0:v>26</ns0:v>
+        <ns0:v>25</ns0:v>
       </ns0:c>
       <ns0:c r="B26" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-06-26</ns0:t>
+          <ns0:t xml:space="preserve">2026-06-29</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C26" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">1ab52989</ns0:t>
+          <ns0:t xml:space="preserve">1a63a634</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D26" s="2" t="inlineStr">
@@ -1911,137 +1911,141 @@
     </ns0:row>
     <ns0:row r="27">
       <ns0:c r="A27" s="0">
+        <ns0:v>26</ns0:v>
+      </ns0:c>
+      <ns0:c r="B27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-07-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">0871bd20</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[ALL]nvmp|cap: Wrap localtime_r/gmtime_r, unify time conversion APIs across NVMP platform[3/4]</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">无差异</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">I2e8c267870f913cae7c1e2d7cbe60251a93656f2</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">将人脸报表的本地时间转换改为 nvmp_localtime_safe，并处理转换失败；与 BC ce7ab9a6 同 Change-Id，但原补丁受各自分支上下文影响，焦点路径 patch-id 不同。当前公共代码的两处转换均使用安全包装。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H27" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I27" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O27" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" s="0">
         <ns0:v>27</ns0:v>
       </ns0:c>
-      <ns0:c r="B27" s="0" t="inlineStr">
+      <ns0:c r="B28" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2026-07-13</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">ebb0da21</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D27" s="0" t="inlineStr">
+      <ns0:c r="C28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">950beb43</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D28" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[ALL] face_snapshot: Fix non-standard code for telemetry support of face recognition</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E27" s="0" t="inlineStr">
+      <ns0:c r="E28" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">编译修复</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F27" s="0" t="inlineStr">
+      <ns0:c r="F28" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">I7dd93f69b756a90ae4b67e4f2573f4c1d20d2ba5</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G27" s="0" t="inlineStr">
+      <ns0:c r="G28" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">修正人脸识别遥测代码的宏边界、空参数返回及接口注册保护，使可选遥测配置下的代码规范且可编译。</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="H27" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I27" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O27" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="28">
-      <ns0:c r="A28" s="2">
-        <ns0:v>28</ns0:v>
-      </ns0:c>
-      <ns0:c r="B28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">2026-07-27</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="C28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">dd2600fb</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap:Add camera log (3/4)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="E28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">跨模块功能</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="F28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">I546ddacdc3c963356cab324458b2e295a1b62e66</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="G28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">在人脸快照配置链中接入摄像机操作日志，记录相关配置动作；属于跨模块系列的 CAP 部分。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H28" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I28" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J28" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K28" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N28" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O28" s="2" t="inlineStr">
+      <ns0:c r="H28" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I28" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N28" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O28" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -2049,21 +2053,21 @@
     </ns0:row>
     <ns0:row r="29">
       <ns0:c r="A29" s="2">
-        <ns0:v>29</ns0:v>
+        <ns0:v>28</ns0:v>
       </ns0:c>
       <ns0:c r="B29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-08-14</ns0:t>
+          <ns0:t xml:space="preserve">2026-07-13</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">14378dec</ns0:t>
+          <ns0:t xml:space="preserve">bf5b7403</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap: modify pre_set method(2/2)</ns0:t>
+          <ns0:t xml:space="preserve">[ALL] cap:Add camera log (3/4)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E29" s="2" t="inlineStr">
@@ -2073,12 +2077,12 @@
       </ns0:c>
       <ns0:c r="F29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Iaf8476f2cb5fc327339218e1cf59a10f865c9bd7</ns0:t>
+          <ns0:t xml:space="preserve">I546ddacdc3c963356cab324458b2e295a1b62e66</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">调整摄像机操作日志相关配置的预设置方法，使配置变更和日志链一致；需结合系列其他模块评审。</ns0:t>
+          <ns0:t xml:space="preserve">在人脸快照配置链中接入摄像机操作日志，记录相关配置动作；属于跨模块系列的 CAP 部分。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H29" s="2">
@@ -2115,77 +2119,144 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="30">
-      <ns0:c r="A30" s="0">
+      <ns0:c r="A30" s="2">
+        <ns0:v>29</ns0:v>
+      </ns0:c>
+      <ns0:c r="B30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-08-14</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">71eef458</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">[Models with CAMERA_OPERATION_LOG_SUPPORT] cap: modify pre_set method(2/2)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">跨模块功能</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Iaf8476f2cb5fc327339218e1cf59a10f865c9bd7</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">调整摄像机操作日志相关配置的预设置方法，使配置变更和日志链一致；需结合系列其他模块评审。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H30" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="I30" s="2">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="J30" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K30" s="2">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O30" s="2" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" s="0">
         <ns0:v>30</ns0:v>
       </ns0:c>
-      <ns0:c r="B30" s="0" t="inlineStr">
+      <ns0:c r="B31" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2026-09-21</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C30" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">178f33f6</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D30" s="0" t="inlineStr">
+      <ns0:c r="C31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">f7d6f0ea</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D31" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[all]cap:Fixed the error in determining the fd in err_exit</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E30" s="0" t="inlineStr">
+      <ns0:c r="E31" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Bug修复</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F30" s="0" t="inlineStr">
+      <ns0:c r="F31" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Ia28fea5b1b63f8146d857ecbcff25f66326e1041</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G30" s="0" t="inlineStr">
+      <ns0:c r="G31" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">修正 PSS 图片复制函数错误退出时的文件描述符判断，按原提交条件关闭已打开的源文件与目标文件。</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="H30" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="I30" s="0">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="J30" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="K30" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="L30" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M30" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N30" s="0" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O30" s="0" t="inlineStr">
+      <ns0:c r="H31" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I31" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="L31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N31" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O31" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>
-  <ns0:autoFilter ref="A1:O30"/>
+  <ns0:autoFilter ref="A1:O31"/>
 </ns0:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(face_snapshot): record canonical AC trial repairs and review outcomes
</commit_message>
<xml_diff>
--- a/branch_diff/face_snapshot-new/ac侧提交概览.xlsx
+++ b/branch_diff/face_snapshot-new/ac侧提交概览.xlsx
@@ -416,24 +416,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J5" s="2">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K5" s="2">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L5" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (share notification pushable selection)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M5" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">caf63fc24af5daa280c8ea2351dfa53e5fb3bf2d</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N5" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">I9cf5626f78979982072533362f72d60615b8a6f6</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O5" s="2" t="inlineStr">
@@ -767,24 +767,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J10" s="2">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K10" s="2">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L10" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (share platform random source) (3/4)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M10" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">734aee51c6e3a08fe43e7cc31865f2a40c4bfb02</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N10" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">If30e5756a7f1aab23b3279b41c64211dafa4585e</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O10" s="2" t="inlineStr">
@@ -1007,67 +1007,67 @@
       </ns0:c>
     </ns0:row>
     <ns0:row r="14">
-      <ns0:c r="A14" s="2">
+      <ns0:c r="A14" s="0">
         <ns0:v>13</ns0:v>
       </ns0:c>
-      <ns0:c r="B14" s="2" t="inlineStr">
+      <ns0:c r="B14" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">2026-01-16</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="C14" s="2" t="inlineStr">
+      <ns0:c r="C14" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">e69adae6</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D14" s="2" t="inlineStr">
+      <ns0:c r="D14" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">[cap]face_snapshot:fix some bugs of face snapshot</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="E14" s="2" t="inlineStr">
+      <ns0:c r="E14" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">Bug修复,有对标提交</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="F14" s="2" t="inlineStr">
+      <ns0:c r="F14" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve">I5432aabc9ef96b11abea1a28420c783eee21832d</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="G14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve">与 BC 99edff3d 同 Change-Id，六项修复目标一致，均处理 HUB 配置缓存、合并旧人脸删除、队列校验及库满覆盖通知；补丁不逐行相同。AC 的 HUB 告警保留 pushable:0，内部删除额外清理陌生人历史，检测入口兼容 PSS；BC 原补丁沿用无 pushable 的 HUB 格式与自身检测入口。需按最终代码核对这些差异。</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="H14" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="I14" s="2">
-        <ns0:v>1</ns0:v>
-      </ns0:c>
-      <ns0:c r="J14" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="K14" s="2">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-      <ns0:c r="L14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="M14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="N14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t xml:space="preserve"/>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="O14" s="2" t="inlineStr">
+      <ns0:c r="G14" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">与 BC 99edff3d 同 Change-Id，均修正 HUB 配置缓存、旧人脸删除、事件队列及库满覆盖通知。当前试合入分支已共用这些修复；HUB 告警消息路由仍有分歧，单独归于 2900128f 审查。本笔无需新增修复提交。</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H14" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I14" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="J14" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K14" s="0">
+        <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="L14" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="M14" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="N14" s="0" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve"/>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="O14" s="0" t="inlineStr">
         <ns0:is>
           <ns0:t xml:space="preserve"/>
         </ns0:is>
@@ -1185,24 +1185,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J16" s="0">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K16" s="0">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L16" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (gate picture config repair by feature flag) (1/2)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M16" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">8b45439c41449fecd19f0ea6a1113ce2031cc407</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N16" s="0" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">I8bb6cb2ccd0936021995376f21edb6bd12f0fa0f</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O16" s="0" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </ns0:c>
       <ns0:c r="G18" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">调整 HUB 存储代理的人脸消息，补齐 faceid、name 和 alias 等字段，使下游 IoT 转发可识别人脸事件；依赖消费端配套。</ns0:t>
+          <ns0:t xml:space="preserve">HUB 存储代理场景改为仅向 MSGID_ALARM_EXT 发送完整人脸事件，并取消单独的 HUB 推送，配套下游解析 faceid、name、alias。当前 BC 路径仍发送 MSGID_HUB_ALARM，BC 的 NSD cloud_iot.c 监听该消息；直接统一会改变消息消费契约。试合入暂缓，需连同 AVTS/hub_storage 消费端审查。</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="H18" s="2">
@@ -1532,24 +1532,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J21" s="2">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K21" s="2">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L21" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (share libfss query callback registration)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M21" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">482854aab99847f942fd99c1c2945e12dd2a2a65</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N21" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">I2b467313120667aa3be900e6df5e012164ab931f</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O21" s="2" t="inlineStr">
@@ -1883,24 +1883,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J26" s="2">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K26" s="2">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L26" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (share optional face telemetry) (2/3)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M26" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">b768d2840e2b3321d4500c4c216eb678f01047fd</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N26" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">Iff71b699361801dedebc8e8d9bae79f311f2dc6f</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O26" s="2" t="inlineStr">
@@ -2092,24 +2092,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J29" s="2">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K29" s="2">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (share camera operation log hook) (3/4)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">f1f92940f016d37a91cee4ba8bb2220d1e491d89</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N29" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">I4a241138230e3587c92ab0a0b60a3bb4b9af4b5f</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O29" s="2" t="inlineStr">
@@ -2159,24 +2159,24 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="J30" s="2">
-        <ns0:v>0</ns0:v>
+        <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="K30" s="2">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="L30" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">[cap] face_snapshot: remove branch macros (share camera log change filtering) (2/2)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="M30" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">e68b2046f8717306cde5126776ba1fbb928a9a4d</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="N30" s="2" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve"/>
+          <ns0:t xml:space="preserve">I3cbc4210922300dabd31422ddfbcfecac7708c8d</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O30" s="2" t="inlineStr">

</xml_diff>